<commit_message>
Update data — 2026-04-10T17:44:34.169Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -682,7 +682,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -700,12 +700,6 @@
       <c r="E1" t="str">
         <v>archivedProjects</v>
       </c>
-      <c r="F1" t="str">
-        <v>committedAt</v>
-      </c>
-      <c r="G1" t="str">
-        <v>committedFrom</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -723,16 +717,10 @@
       <c r="E2" t="str">
         <v>[]</v>
       </c>
-      <c r="F2" t="str">
-        <v>2026-04-10T17:37:17.781Z</v>
-      </c>
-      <c r="G2" t="str">
-        <v>KneuraCOMMS Landing</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update data — 2026-04-10T17:45:02.380Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,42 +463,42 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>0t32y7xn</v>
+        <v>44wm985n</v>
       </c>
       <c r="B3" t="str">
-        <v>Review Q3 expense report</v>
+        <v>Set up analytics dashboard</v>
       </c>
       <c r="C3" t="str">
-        <v>CFO</v>
+        <v>CIO</v>
       </c>
       <c r="D3" t="str">
-        <v>zw42pfcs</v>
+        <v>1fno5axv</v>
       </c>
       <c r="E3" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>pending</v>
+        <v>blocked</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-09</v>
+        <v>2026-04-11</v>
       </c>
       <c r="H3" t="str">
-        <v>Pull receipts from Notion</v>
+        <v>Unblock API access from vendor</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>Waiting on vendor</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>44wm985n</v>
+        <v>x89mr83u</v>
       </c>
       <c r="B4" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C4" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D4" t="str">
         <v>1fno5axv</v>
@@ -507,50 +507,21 @@
         <v>medium</v>
       </c>
       <c r="F4" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I4" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>x89mr83u</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C5" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D5" t="str">
-        <v>1fno5axv</v>
-      </c>
-      <c r="E5" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F5" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update data — 2026-04-10T17:45:07.528Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,42 +434,42 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>yi6pymud</v>
+        <v>44wm985n</v>
       </c>
       <c r="B2" t="str">
-        <v>Finalize product roadmap</v>
+        <v>Set up analytics dashboard</v>
       </c>
       <c r="C2" t="str">
-        <v>CEO</v>
+        <v>CIO</v>
       </c>
       <c r="D2" t="str">
         <v>1fno5axv</v>
       </c>
       <c r="E2" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v>in-progress</v>
+        <v>blocked</v>
       </c>
       <c r="G2" t="str">
         <v>2026-04-11</v>
       </c>
       <c r="H2" t="str">
-        <v>Write Q4 objectives section</v>
+        <v>Unblock API access from vendor</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>Waiting on vendor</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>44wm985n</v>
+        <v>x89mr83u</v>
       </c>
       <c r="B3" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C3" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D3" t="str">
         <v>1fno5axv</v>
@@ -478,50 +478,21 @@
         <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I3" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>x89mr83u</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C4" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D4" t="str">
-        <v>1fno5axv</v>
-      </c>
-      <c r="E4" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F4" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update data — 2026-04-10T17:45:12.371Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,13 +434,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>44wm985n</v>
+        <v>x89mr83u</v>
       </c>
       <c r="B2" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C2" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D2" t="str">
         <v>1fno5axv</v>
@@ -449,50 +449,21 @@
         <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I2" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>x89mr83u</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D3" t="str">
-        <v>1fno5axv</v>
-      </c>
-      <c r="E3" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F3" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update data — 2026-04-10T17:45:16.517Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>x89mr83u</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Launch email campaign</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>CMO</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>1fno5axv</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>medium</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>pending</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>Draft campaign brief</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>

</xml_diff>

<commit_message>
KneuraCOMMS commit — 2026-04-10T17:48:17.688Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,36 +434,123 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>iu4dha0q</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Finalize product roadmap</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>3j9y1njh</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>high</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>in-progress</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-04-11</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>Write Q4 objectives section</v>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>b25kb7up</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Review Q3 expense report</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>j743noye</v>
+      </c>
+      <c r="E3" t="str">
+        <v>high</v>
+      </c>
+      <c r="F3" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-04-09</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Pull receipts from Notion</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>dseebszz</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Set up analytics dashboard</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CIO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>3j9y1njh</v>
+      </c>
+      <c r="E4" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F4" t="str">
+        <v>blocked</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Unblock API access from vendor</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Waiting on vendor</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>pj7epeho</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Launch email campaign</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CMO</v>
+      </c>
+      <c r="D5" t="str">
+        <v>3j9y1njh</v>
+      </c>
+      <c r="E5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F5" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Draft campaign brief</v>
+      </c>
+      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -488,7 +575,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1fno5axv</v>
+        <v>3j9y1njh</v>
       </c>
       <c r="B2" t="str">
         <v>Product Launch</v>
@@ -502,7 +589,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>zw42pfcs</v>
+        <v>j743noye</v>
       </c>
       <c r="B3" t="str">
         <v>Q3 Financials</v>

</xml_diff>

<commit_message>
Update data — 2026-04-10T17:48:28.463Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,42 +463,42 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>b25kb7up</v>
+        <v>dseebszz</v>
       </c>
       <c r="B3" t="str">
-        <v>Review Q3 expense report</v>
+        <v>Set up analytics dashboard</v>
       </c>
       <c r="C3" t="str">
-        <v>CFO</v>
+        <v>CIO</v>
       </c>
       <c r="D3" t="str">
-        <v>j743noye</v>
+        <v>3j9y1njh</v>
       </c>
       <c r="E3" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>pending</v>
+        <v>blocked</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-09</v>
+        <v>2026-04-11</v>
       </c>
       <c r="H3" t="str">
-        <v>Pull receipts from Notion</v>
+        <v>Unblock API access from vendor</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>Waiting on vendor</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>dseebszz</v>
+        <v>pj7epeho</v>
       </c>
       <c r="B4" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C4" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D4" t="str">
         <v>3j9y1njh</v>
@@ -507,50 +507,21 @@
         <v>medium</v>
       </c>
       <c r="F4" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I4" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>pj7epeho</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C5" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D5" t="str">
-        <v>3j9y1njh</v>
-      </c>
-      <c r="E5" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F5" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update data — 2026-04-10T17:48:32.339Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,42 +434,42 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>iu4dha0q</v>
+        <v>dseebszz</v>
       </c>
       <c r="B2" t="str">
-        <v>Finalize product roadmap</v>
+        <v>Set up analytics dashboard</v>
       </c>
       <c r="C2" t="str">
-        <v>CEO</v>
+        <v>CIO</v>
       </c>
       <c r="D2" t="str">
         <v>3j9y1njh</v>
       </c>
       <c r="E2" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v>in-progress</v>
+        <v>blocked</v>
       </c>
       <c r="G2" t="str">
         <v>2026-04-11</v>
       </c>
       <c r="H2" t="str">
-        <v>Write Q4 objectives section</v>
+        <v>Unblock API access from vendor</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>Waiting on vendor</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>dseebszz</v>
+        <v>pj7epeho</v>
       </c>
       <c r="B3" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C3" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D3" t="str">
         <v>3j9y1njh</v>
@@ -478,50 +478,21 @@
         <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I3" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>pj7epeho</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C4" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D4" t="str">
-        <v>3j9y1njh</v>
-      </c>
-      <c r="E4" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F4" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update data — 2026-04-10T17:48:36.626Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -461,38 +461,9 @@
         <v>Waiting on vendor</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>pj7epeho</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D3" t="str">
-        <v>3j9y1njh</v>
-      </c>
-      <c r="E3" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F3" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update data — 2026-04-10T17:48:42.399Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,31 +434,31 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>dseebszz</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Set up analytics dashboard</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>CIO</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>3j9y1njh</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>medium</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>blocked</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>Unblock API access from vendor</v>
+        <v/>
       </c>
       <c r="I2" t="str">
-        <v>Waiting on vendor</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T17:59:50.355Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>24a67n8j</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>TEst</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>CEO</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>pending</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-04-10</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>test</v>
       </c>
       <c r="I2" t="str">
         <v/>

</xml_diff>

<commit_message>
Update data — 2026-04-10T18:00:07.820Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>24a67n8j</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>TEst</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>CEO</v>
+        <v/>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>medium</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>done</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-10</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>test</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>

</xml_diff>

<commit_message>
Update data — 2026-04-10T18:29:24.262Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -595,7 +595,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -613,6 +613,9 @@
       <c r="E1" t="str">
         <v>archivedProjects</v>
       </c>
+      <c r="F1" t="str">
+        <v>savedAt</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -630,10 +633,13 @@
       <c r="E2" t="str">
         <v>[]</v>
       </c>
+      <c r="F2" t="str">
+        <v>2026-04-10T18:29:24.223Z</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update data — 2026-04-10T18:29:51.113Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -470,7 +470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -514,9 +514,23 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>wjbb9ft4</v>
+      </c>
+      <c r="B4" t="str">
+        <v>TerraIntel360</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CEO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Agritourism Project by Roots &amp; Routes LLC</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -634,7 +648,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T18:29:24.223Z</v>
+        <v>2026-04-10T18:29:51.092Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T18:30:05.050Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -470,7 +470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,13 +488,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>3j9y1njh</v>
+        <v>j743noye</v>
       </c>
       <c r="B2" t="str">
-        <v>Product Launch</v>
+        <v>Q3 Financials</v>
       </c>
       <c r="C2" t="str">
-        <v>CEO</v>
+        <v>CFO</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -502,35 +502,21 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>j743noye</v>
+        <v>wjbb9ft4</v>
       </c>
       <c r="B3" t="str">
-        <v>Q3 Financials</v>
+        <v>TerraIntel360</v>
       </c>
       <c r="C3" t="str">
-        <v>CFO</v>
+        <v>CEO</v>
       </c>
       <c r="D3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>wjbb9ft4</v>
-      </c>
-      <c r="B4" t="str">
-        <v>TerraIntel360</v>
-      </c>
-      <c r="C4" t="str">
-        <v>CEO</v>
-      </c>
-      <c r="D4" t="str">
         <v>Agritourism Project by Roots &amp; Routes LLC</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -648,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T18:29:54.223Z</v>
+        <v>2026-04-10T18:30:05.029Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T18:30:11.055Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -470,7 +470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,35 +488,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>j743noye</v>
+        <v>wjbb9ft4</v>
       </c>
       <c r="B2" t="str">
-        <v>Q3 Financials</v>
+        <v>TerraIntel360</v>
       </c>
       <c r="C2" t="str">
-        <v>CFO</v>
+        <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>wjbb9ft4</v>
-      </c>
-      <c r="B3" t="str">
-        <v>TerraIntel360</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CEO</v>
-      </c>
-      <c r="D3" t="str">
         <v>Agritourism Project by Roots &amp; Routes LLC</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -634,7 +620,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T18:30:05.029Z</v>
+        <v>2026-04-10T18:30:11.038Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T18:32:00.424Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,31 +434,31 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>gsk1oc9f</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Close the deal. Get a Contract</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>wjbb9ft4</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>in-progress</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-06-30</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>Talk to her about the funding progress</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>Currently Tracy is exploring fundings</v>
       </c>
     </row>
   </sheetData>
@@ -620,7 +620,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T18:31:54.222Z</v>
+        <v>2026-04-10T18:32:00.411Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KneuraCOMMS commit — 2026-04-10T21:27:03.000Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,43 +434,130 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>gsk1oc9f</v>
+        <v>xhcfhezw</v>
       </c>
       <c r="B2" t="str">
-        <v>Close the deal. Get a Contract</v>
+        <v>Finalize product roadmap</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v>wjbb9ft4</v>
+        <v>vrx2qf6c</v>
       </c>
       <c r="E2" t="str">
-        <v>medium</v>
+        <v>high</v>
       </c>
       <c r="F2" t="str">
         <v>in-progress</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-06-30</v>
+        <v>2026-04-11</v>
       </c>
       <c r="H2" t="str">
-        <v>Talk to her about the funding progress</v>
+        <v>Write Q4 objectives section</v>
       </c>
       <c r="I2" t="str">
-        <v>Currently Tracy is exploring fundings</v>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>x03eaa3b</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Review Q3 expense report</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>suvyo3kt</v>
+      </c>
+      <c r="E3" t="str">
+        <v>high</v>
+      </c>
+      <c r="F3" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-04-09</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Pull receipts from Notion</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>gzlpb1kc</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Set up analytics dashboard</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CIO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>vrx2qf6c</v>
+      </c>
+      <c r="E4" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F4" t="str">
+        <v>blocked</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Unblock API access from vendor</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Waiting on vendor</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>3nftmans</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Launch email campaign</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CMO</v>
+      </c>
+      <c r="D5" t="str">
+        <v>vrx2qf6c</v>
+      </c>
+      <c r="E5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F5" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Draft campaign brief</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,21 +575,35 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>wjbb9ft4</v>
+        <v>vrx2qf6c</v>
       </c>
       <c r="B2" t="str">
-        <v>TerraIntel360</v>
+        <v>Product Launch</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v>Agritourism Project by Roots &amp; Routes LLC</v>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>suvyo3kt</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Q3 Financials</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -620,7 +721,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T20:16:22.507Z</v>
+        <v>2026-04-10T21:27:02.284Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:27:18.485Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,42 +463,42 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>x03eaa3b</v>
+        <v>gzlpb1kc</v>
       </c>
       <c r="B3" t="str">
-        <v>Review Q3 expense report</v>
+        <v>Set up analytics dashboard</v>
       </c>
       <c r="C3" t="str">
-        <v>CFO</v>
+        <v>CIO</v>
       </c>
       <c r="D3" t="str">
-        <v>suvyo3kt</v>
+        <v>vrx2qf6c</v>
       </c>
       <c r="E3" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>pending</v>
+        <v>blocked</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-09</v>
+        <v>2026-04-11</v>
       </c>
       <c r="H3" t="str">
-        <v>Pull receipts from Notion</v>
+        <v>Unblock API access from vendor</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>Waiting on vendor</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>gzlpb1kc</v>
+        <v>3nftmans</v>
       </c>
       <c r="B4" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C4" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D4" t="str">
         <v>vrx2qf6c</v>
@@ -507,50 +507,21 @@
         <v>medium</v>
       </c>
       <c r="F4" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I4" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>3nftmans</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C5" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D5" t="str">
-        <v>vrx2qf6c</v>
-      </c>
-      <c r="E5" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F5" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -721,7 +692,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:27:02.284Z</v>
+        <v>2026-04-10T21:27:18.460Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:27:21.943Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,13 +463,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>gzlpb1kc</v>
+        <v>3nftmans</v>
       </c>
       <c r="B3" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C3" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D3" t="str">
         <v>vrx2qf6c</v>
@@ -478,50 +478,21 @@
         <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I3" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>3nftmans</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C4" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D4" t="str">
-        <v>vrx2qf6c</v>
-      </c>
-      <c r="E4" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F4" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -692,7 +663,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:27:18.460Z</v>
+        <v>2026-04-10T21:27:21.937Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:27:28.329Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,65 +434,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>xhcfhezw</v>
+        <v>3nftmans</v>
       </c>
       <c r="B2" t="str">
-        <v>Finalize product roadmap</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C2" t="str">
-        <v>CEO</v>
+        <v>CMO</v>
       </c>
       <c r="D2" t="str">
         <v>vrx2qf6c</v>
       </c>
       <c r="E2" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v>in-progress</v>
+        <v>pending</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>Write Q4 objectives section</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>3nftmans</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D3" t="str">
-        <v>vrx2qf6c</v>
-      </c>
-      <c r="E3" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F3" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -663,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:27:21.937Z</v>
+        <v>2026-04-10T21:27:28.310Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:27:33.557Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>3nftmans</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Launch email campaign</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>CMO</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>vrx2qf6c</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>medium</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>pending</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>Draft campaign brief</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -634,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:27:30.670Z</v>
+        <v>2026-04-10T21:27:33.544Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:28:49.941Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,36 +434,123 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>xhcfhezw</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Finalize product roadmap</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>vrx2qf6c</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>high</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>in-progress</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-04-11</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>Write Q4 objectives section</v>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>x03eaa3b</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Review Q3 expense report</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>suvyo3kt</v>
+      </c>
+      <c r="E3" t="str">
+        <v>high</v>
+      </c>
+      <c r="F3" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-04-09</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Pull receipts from Notion</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>gzlpb1kc</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Set up analytics dashboard</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CIO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>vrx2qf6c</v>
+      </c>
+      <c r="E4" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F4" t="str">
+        <v>blocked</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Unblock API access from vendor</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Waiting on vendor</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>3nftmans</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Launch email campaign</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CMO</v>
+      </c>
+      <c r="D5" t="str">
+        <v>vrx2qf6c</v>
+      </c>
+      <c r="E5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F5" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Draft campaign brief</v>
+      </c>
+      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -634,7 +721,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:27:46.921Z</v>
+        <v>2026-04-10T21:28:49.923Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:28:57.224Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,42 +463,42 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>x03eaa3b</v>
+        <v>gzlpb1kc</v>
       </c>
       <c r="B3" t="str">
-        <v>Review Q3 expense report</v>
+        <v>Set up analytics dashboard</v>
       </c>
       <c r="C3" t="str">
-        <v>CFO</v>
+        <v>CIO</v>
       </c>
       <c r="D3" t="str">
-        <v>suvyo3kt</v>
+        <v>vrx2qf6c</v>
       </c>
       <c r="E3" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>pending</v>
+        <v>blocked</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-09</v>
+        <v>2026-04-11</v>
       </c>
       <c r="H3" t="str">
-        <v>Pull receipts from Notion</v>
+        <v>Unblock API access from vendor</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>Waiting on vendor</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>gzlpb1kc</v>
+        <v>3nftmans</v>
       </c>
       <c r="B4" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C4" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D4" t="str">
         <v>vrx2qf6c</v>
@@ -507,50 +507,21 @@
         <v>medium</v>
       </c>
       <c r="F4" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I4" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>3nftmans</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C5" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D5" t="str">
-        <v>vrx2qf6c</v>
-      </c>
-      <c r="E5" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F5" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -721,7 +692,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:28:49.923Z</v>
+        <v>2026-04-10T21:28:57.220Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:29:02.691Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,13 +463,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>gzlpb1kc</v>
+        <v>3nftmans</v>
       </c>
       <c r="B3" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C3" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D3" t="str">
         <v>vrx2qf6c</v>
@@ -478,50 +478,21 @@
         <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I3" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>3nftmans</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C4" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D4" t="str">
-        <v>vrx2qf6c</v>
-      </c>
-      <c r="E4" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F4" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -692,7 +663,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:28:57.220Z</v>
+        <v>2026-04-10T21:29:02.672Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:29:07.269Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,65 +434,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>xhcfhezw</v>
+        <v>3nftmans</v>
       </c>
       <c r="B2" t="str">
-        <v>Finalize product roadmap</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C2" t="str">
-        <v>CEO</v>
+        <v>CMO</v>
       </c>
       <c r="D2" t="str">
         <v>vrx2qf6c</v>
       </c>
       <c r="E2" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v>in-progress</v>
+        <v>pending</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>Write Q4 objectives section</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>3nftmans</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D3" t="str">
-        <v>vrx2qf6c</v>
-      </c>
-      <c r="E3" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F3" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -663,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:29:02.672Z</v>
+        <v>2026-04-10T21:29:07.258Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:29:12.187Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>3nftmans</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Launch email campaign</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>CMO</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>vrx2qf6c</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>medium</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>pending</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>Draft campaign brief</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -634,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:29:07.258Z</v>
+        <v>2026-04-10T21:29:12.170Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KneuraCOMMS commit — 2026-04-10T21:30:08.566Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,36 +434,123 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>xhcfhezw</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Finalize product roadmap</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>vrx2qf6c</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>high</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>in-progress</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-04-11</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>Write Q4 objectives section</v>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>x03eaa3b</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Review Q3 expense report</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>suvyo3kt</v>
+      </c>
+      <c r="E3" t="str">
+        <v>high</v>
+      </c>
+      <c r="F3" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-04-09</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Pull receipts from Notion</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>gzlpb1kc</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Set up analytics dashboard</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CIO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>vrx2qf6c</v>
+      </c>
+      <c r="E4" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F4" t="str">
+        <v>blocked</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Unblock API access from vendor</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Waiting on vendor</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>3nftmans</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Launch email campaign</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CMO</v>
+      </c>
+      <c r="D5" t="str">
+        <v>vrx2qf6c</v>
+      </c>
+      <c r="E5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F5" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Draft campaign brief</v>
+      </c>
+      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -634,7 +721,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:29:40.416Z</v>
+        <v>2026-04-10T21:30:08.157Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:30:34.096Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,42 +463,42 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>x03eaa3b</v>
+        <v>gzlpb1kc</v>
       </c>
       <c r="B3" t="str">
-        <v>Review Q3 expense report</v>
+        <v>Set up analytics dashboard</v>
       </c>
       <c r="C3" t="str">
-        <v>CFO</v>
+        <v>CIO</v>
       </c>
       <c r="D3" t="str">
-        <v>suvyo3kt</v>
+        <v>vrx2qf6c</v>
       </c>
       <c r="E3" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>pending</v>
+        <v>blocked</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-09</v>
+        <v>2026-04-11</v>
       </c>
       <c r="H3" t="str">
-        <v>Pull receipts from Notion</v>
+        <v>Unblock API access from vendor</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>Waiting on vendor</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>gzlpb1kc</v>
+        <v>3nftmans</v>
       </c>
       <c r="B4" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C4" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D4" t="str">
         <v>vrx2qf6c</v>
@@ -507,50 +507,21 @@
         <v>medium</v>
       </c>
       <c r="F4" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I4" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>3nftmans</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C5" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D5" t="str">
-        <v>vrx2qf6c</v>
-      </c>
-      <c r="E5" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F5" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -721,7 +692,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:30:27.479Z</v>
+        <v>2026-04-10T21:30:34.073Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:30:38.565Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,13 +463,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>gzlpb1kc</v>
+        <v>3nftmans</v>
       </c>
       <c r="B3" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C3" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D3" t="str">
         <v>vrx2qf6c</v>
@@ -478,50 +478,21 @@
         <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I3" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>3nftmans</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C4" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D4" t="str">
-        <v>vrx2qf6c</v>
-      </c>
-      <c r="E4" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F4" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -692,7 +663,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:30:34.073Z</v>
+        <v>2026-04-10T21:30:38.544Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:30:42.288Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,65 +434,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>xhcfhezw</v>
+        <v>3nftmans</v>
       </c>
       <c r="B2" t="str">
-        <v>Finalize product roadmap</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C2" t="str">
-        <v>CEO</v>
+        <v>CMO</v>
       </c>
       <c r="D2" t="str">
         <v>vrx2qf6c</v>
       </c>
       <c r="E2" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v>in-progress</v>
+        <v>pending</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>Write Q4 objectives section</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>3nftmans</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D3" t="str">
-        <v>vrx2qf6c</v>
-      </c>
-      <c r="E3" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F3" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -663,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:30:38.544Z</v>
+        <v>2026-04-10T21:30:42.276Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:30:46.419Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>3nftmans</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Launch email campaign</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>CMO</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>vrx2qf6c</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>medium</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>pending</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>Draft campaign brief</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -634,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:30:42.276Z</v>
+        <v>2026-04-10T21:30:46.404Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KneuraCOMMS commit — 2026-04-10T21:31:40.109Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,36 +434,123 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>fslsfdan</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Finalize product roadmap</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>am6wy3t6</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>high</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>in-progress</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-04-11</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>Write Q4 objectives section</v>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>91dr2ciu</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Review Q3 expense report</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>c7dpc4r1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>high</v>
+      </c>
+      <c r="F3" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-04-09</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Pull receipts from Notion</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>0hwz5cax</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Set up analytics dashboard</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CIO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>am6wy3t6</v>
+      </c>
+      <c r="E4" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F4" t="str">
+        <v>blocked</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Unblock API access from vendor</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Waiting on vendor</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>olh24ydv</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Launch email campaign</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CMO</v>
+      </c>
+      <c r="D5" t="str">
+        <v>am6wy3t6</v>
+      </c>
+      <c r="E5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F5" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Draft campaign brief</v>
+      </c>
+      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -488,7 +575,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>vrx2qf6c</v>
+        <v>am6wy3t6</v>
       </c>
       <c r="B2" t="str">
         <v>Product Launch</v>
@@ -502,7 +589,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>suvyo3kt</v>
+        <v>c7dpc4r1</v>
       </c>
       <c r="B3" t="str">
         <v>Q3 Financials</v>
@@ -634,7 +721,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:30:59.664Z</v>
+        <v>2026-04-10T21:31:39.415Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:31:54.373Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,42 +463,42 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>91dr2ciu</v>
+        <v>0hwz5cax</v>
       </c>
       <c r="B3" t="str">
-        <v>Review Q3 expense report</v>
+        <v>Set up analytics dashboard</v>
       </c>
       <c r="C3" t="str">
-        <v>CFO</v>
+        <v>CIO</v>
       </c>
       <c r="D3" t="str">
-        <v>c7dpc4r1</v>
+        <v>am6wy3t6</v>
       </c>
       <c r="E3" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>pending</v>
+        <v>blocked</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-09</v>
+        <v>2026-04-11</v>
       </c>
       <c r="H3" t="str">
-        <v>Pull receipts from Notion</v>
+        <v>Unblock API access from vendor</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>Waiting on vendor</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>0hwz5cax</v>
+        <v>olh24ydv</v>
       </c>
       <c r="B4" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C4" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D4" t="str">
         <v>am6wy3t6</v>
@@ -507,50 +507,21 @@
         <v>medium</v>
       </c>
       <c r="F4" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I4" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>olh24ydv</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C5" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D5" t="str">
-        <v>am6wy3t6</v>
-      </c>
-      <c r="E5" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F5" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -721,7 +692,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:31:43.644Z</v>
+        <v>2026-04-10T21:31:54.361Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:31:57.245Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,13 +463,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>0hwz5cax</v>
+        <v>olh24ydv</v>
       </c>
       <c r="B3" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C3" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D3" t="str">
         <v>am6wy3t6</v>
@@ -478,50 +478,21 @@
         <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I3" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>olh24ydv</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C4" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D4" t="str">
-        <v>am6wy3t6</v>
-      </c>
-      <c r="E4" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F4" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -692,7 +663,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:31:54.361Z</v>
+        <v>2026-04-10T21:31:57.221Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KneuraCOMMS commit — 2026-04-10T21:33:07.262Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,72 +434,43 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>fslsfdan</v>
+        <v>2aru55my</v>
       </c>
       <c r="B2" t="str">
-        <v>Finalize product roadmap</v>
+        <v>Get the Project Onboard</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v>am6wy3t6</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v>in-progress</v>
+        <v>pending</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-11</v>
+        <v>2026-04-10</v>
       </c>
       <c r="H2" t="str">
-        <v>Write Q4 objectives section</v>
+        <v>Talk to Tracy M Griggs</v>
       </c>
       <c r="I2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>olh24ydv</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D3" t="str">
-        <v>am6wy3t6</v>
-      </c>
-      <c r="E3" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F3" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -517,35 +488,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>am6wy3t6</v>
+        <v>1o29wv8l</v>
       </c>
       <c r="B2" t="str">
-        <v>Product Launch</v>
+        <v>TerraIntel360</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>c7dpc4r1</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Q3 Financials</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CFO</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
+        <v>Agritourism Portal for Roots &amp; Routes LLC</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -660,10 +617,10 @@
         <v>{}</v>
       </c>
       <c r="E2" t="str">
-        <v>[]</v>
+        <v>[{"id":"le44qgsv","name":"Product Launch","role":"CEO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"},{"id":"ufmxr0yx","name":"Q3 Financials","role":"CFO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"}]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:33:04.972Z</v>
+        <v>2026-04-10T21:33:06.422Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:33:32.371Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,43 +434,72 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2aru55my</v>
+        <v>fslsfdan</v>
       </c>
       <c r="B2" t="str">
-        <v>Get the Project Onboard</v>
+        <v>Finalize product roadmap</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>am6wy3t6</v>
       </c>
       <c r="E2" t="str">
+        <v>high</v>
+      </c>
+      <c r="F2" t="str">
+        <v>in-progress</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Write Q4 objectives section</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>olh24ydv</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Launch email campaign</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CMO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>am6wy3t6</v>
+      </c>
+      <c r="E3" t="str">
         <v>medium</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F3" t="str">
         <v>pending</v>
       </c>
-      <c r="G2" t="str">
-        <v>2026-04-10</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Talk to Tracy M Griggs</v>
-      </c>
-      <c r="I2" t="str">
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>Draft campaign brief</v>
+      </c>
+      <c r="I3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,21 +517,35 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1o29wv8l</v>
+        <v>am6wy3t6</v>
       </c>
       <c r="B2" t="str">
-        <v>TerraIntel360</v>
+        <v>Product Launch</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v>Agritourism Portal for Roots &amp; Routes LLC</v>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>c7dpc4r1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Q3 Financials</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -617,10 +660,10 @@
         <v>{}</v>
       </c>
       <c r="E2" t="str">
-        <v>[{"id":"le44qgsv","name":"Product Launch","role":"CEO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"},{"id":"ufmxr0yx","name":"Q3 Financials","role":"CFO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"}]</v>
+        <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:33:20.670Z</v>
+        <v>2026-04-10T21:33:32.359Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:33:36.266Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -449,7 +449,7 @@
         <v>high</v>
       </c>
       <c r="F2" t="str">
-        <v>in-progress</v>
+        <v>done</v>
       </c>
       <c r="G2" t="str">
         <v>2026-04-11</v>
@@ -663,7 +663,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:33:32.359Z</v>
+        <v>2026-04-10T21:33:36.246Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:33:45.515Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,65 +434,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>fslsfdan</v>
+        <v>olh24ydv</v>
       </c>
       <c r="B2" t="str">
-        <v>Finalize product roadmap</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C2" t="str">
-        <v>CEO</v>
+        <v>CMO</v>
       </c>
       <c r="D2" t="str">
         <v>am6wy3t6</v>
       </c>
       <c r="E2" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v>done</v>
+        <v>pending</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>Write Q4 objectives section</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>olh24ydv</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D3" t="str">
-        <v>am6wy3t6</v>
-      </c>
-      <c r="E3" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F3" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -663,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:33:36.246Z</v>
+        <v>2026-04-10T21:33:45.496Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:33:51.761Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>olh24ydv</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Launch email campaign</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>CMO</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>am6wy3t6</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>medium</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>pending</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>Draft campaign brief</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -634,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:33:45.496Z</v>
+        <v>2026-04-10T21:33:51.743Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:34:02.241Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>2aru55my</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Get the Project Onboard</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>CEO</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>pending</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-04-10</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>Talk to Tracy M Griggs</v>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -470,7 +470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,35 +488,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>am6wy3t6</v>
+        <v>1o29wv8l</v>
       </c>
       <c r="B2" t="str">
-        <v>Product Launch</v>
+        <v>TerraIntel360</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>c7dpc4r1</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Q3 Financials</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CFO</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
+        <v>Agritourism Portal for Roots &amp; Routes LLC</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -631,10 +617,10 @@
         <v>{}</v>
       </c>
       <c r="E2" t="str">
-        <v>[]</v>
+        <v>[{"id":"le44qgsv","name":"Product Launch","role":"CEO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"},{"id":"ufmxr0yx","name":"Q3 Financials","role":"CFO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"}]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:33:56.018Z</v>
+        <v>2026-04-10T21:34:02.232Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:34:48.337Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2aru55my</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Get the Project Onboard</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>CEO</v>
+        <v/>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>medium</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>pending</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-10</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>Talk to Tracy M Griggs</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -470,7 +470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,21 +488,35 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1o29wv8l</v>
+        <v>am6wy3t6</v>
       </c>
       <c r="B2" t="str">
-        <v>TerraIntel360</v>
+        <v>Product Launch</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v>Agritourism Portal for Roots &amp; Routes LLC</v>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>c7dpc4r1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Q3 Financials</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -617,10 +631,10 @@
         <v>{}</v>
       </c>
       <c r="E2" t="str">
-        <v>[{"id":"le44qgsv","name":"Product Launch","role":"CEO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"},{"id":"ufmxr0yx","name":"Q3 Financials","role":"CFO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"}]</v>
+        <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:34:34.025Z</v>
+        <v>2026-04-10T21:34:48.316Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:35:36.852Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>2aru55my</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Get the Project Onboard</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>CEO</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>pending</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-04-10</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>Talk to Tracy M Griggs</v>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -470,7 +470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,35 +488,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>am6wy3t6</v>
+        <v>1o29wv8l</v>
       </c>
       <c r="B2" t="str">
-        <v>Product Launch</v>
+        <v>TerraIntel360</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>c7dpc4r1</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Q3 Financials</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CFO</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
+        <v>Agritourism Portal for Roots &amp; Routes LLC</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -631,10 +617,10 @@
         <v>{}</v>
       </c>
       <c r="E2" t="str">
-        <v>[]</v>
+        <v>[{"id":"le44qgsv","name":"Product Launch","role":"CEO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"},{"id":"ufmxr0yx","name":"Q3 Financials","role":"CFO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"}]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:34:54.116Z</v>
+        <v>2026-04-10T21:35:36.827Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KneuraCOMMS commit — 2026-04-10T21:36:22.296Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,43 +434,130 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2aru55my</v>
+        <v>rxhwjdja</v>
       </c>
       <c r="B2" t="str">
-        <v>Get the Project Onboard</v>
+        <v>Finalize product roadmap</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>gtvjoxp5</v>
       </c>
       <c r="E2" t="str">
+        <v>high</v>
+      </c>
+      <c r="F2" t="str">
+        <v>in-progress</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Write Q4 objectives section</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>xurewhsr</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Review Q3 expense report</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>fqfexnca</v>
+      </c>
+      <c r="E3" t="str">
+        <v>high</v>
+      </c>
+      <c r="F3" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-04-09</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Pull receipts from Notion</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>jw2l1lr8</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Set up analytics dashboard</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CIO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>gtvjoxp5</v>
+      </c>
+      <c r="E4" t="str">
         <v>medium</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F4" t="str">
+        <v>blocked</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Unblock API access from vendor</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Waiting on vendor</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>mp9laie6</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Launch email campaign</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CMO</v>
+      </c>
+      <c r="D5" t="str">
+        <v>gtvjoxp5</v>
+      </c>
+      <c r="E5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F5" t="str">
         <v>pending</v>
       </c>
-      <c r="G2" t="str">
-        <v>2026-04-10</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Talk to Tracy M Griggs</v>
-      </c>
-      <c r="I2" t="str">
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Draft campaign brief</v>
+      </c>
+      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,21 +575,35 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1o29wv8l</v>
+        <v>gtvjoxp5</v>
       </c>
       <c r="B2" t="str">
-        <v>TerraIntel360</v>
+        <v>Product Launch</v>
       </c>
       <c r="C2" t="str">
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v>Agritourism Portal for Roots &amp; Routes LLC</v>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>fqfexnca</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Q3 Financials</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -617,10 +718,10 @@
         <v>{}</v>
       </c>
       <c r="E2" t="str">
-        <v>[{"id":"le44qgsv","name":"Product Launch","role":"CEO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"},{"id":"ufmxr0yx","name":"Q3 Financials","role":"CFO","desc":"","archivedAt":"2026-04-10T12:50:23.225Z"}]</v>
+        <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:35:36.827Z</v>
+        <v>2026-04-10T21:36:21.488Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:36:35.946Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,42 +463,42 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>xurewhsr</v>
+        <v>jw2l1lr8</v>
       </c>
       <c r="B3" t="str">
-        <v>Review Q3 expense report</v>
+        <v>Set up analytics dashboard</v>
       </c>
       <c r="C3" t="str">
-        <v>CFO</v>
+        <v>CIO</v>
       </c>
       <c r="D3" t="str">
-        <v>fqfexnca</v>
+        <v>gtvjoxp5</v>
       </c>
       <c r="E3" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>pending</v>
+        <v>blocked</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-09</v>
+        <v>2026-04-11</v>
       </c>
       <c r="H3" t="str">
-        <v>Pull receipts from Notion</v>
+        <v>Unblock API access from vendor</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>Waiting on vendor</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>jw2l1lr8</v>
+        <v>mp9laie6</v>
       </c>
       <c r="B4" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C4" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D4" t="str">
         <v>gtvjoxp5</v>
@@ -507,50 +507,21 @@
         <v>medium</v>
       </c>
       <c r="F4" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I4" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>mp9laie6</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C5" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D5" t="str">
-        <v>gtvjoxp5</v>
-      </c>
-      <c r="E5" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F5" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -721,7 +692,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:36:30.189Z</v>
+        <v>2026-04-10T21:36:35.941Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:36:44.366Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,13 +463,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>jw2l1lr8</v>
+        <v>mp9laie6</v>
       </c>
       <c r="B3" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C3" t="str">
-        <v>CIO</v>
+        <v>CMO</v>
       </c>
       <c r="D3" t="str">
         <v>gtvjoxp5</v>
@@ -478,50 +478,21 @@
         <v>medium</v>
       </c>
       <c r="F3" t="str">
-        <v>blocked</v>
+        <v>pending</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I3" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>mp9laie6</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C4" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D4" t="str">
-        <v>gtvjoxp5</v>
-      </c>
-      <c r="E4" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F4" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -692,7 +663,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:36:35.941Z</v>
+        <v>2026-04-10T21:36:44.359Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:36:48.268Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,65 +434,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>rxhwjdja</v>
+        <v>mp9laie6</v>
       </c>
       <c r="B2" t="str">
-        <v>Finalize product roadmap</v>
+        <v>Launch email campaign</v>
       </c>
       <c r="C2" t="str">
-        <v>CEO</v>
+        <v>CMO</v>
       </c>
       <c r="D2" t="str">
         <v>gtvjoxp5</v>
       </c>
       <c r="E2" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="F2" t="str">
-        <v>in-progress</v>
+        <v>pending</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-11</v>
+        <v/>
       </c>
       <c r="H2" t="str">
-        <v>Write Q4 objectives section</v>
+        <v>Draft campaign brief</v>
       </c>
       <c r="I2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>mp9laie6</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D3" t="str">
-        <v>gtvjoxp5</v>
-      </c>
-      <c r="E3" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F3" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -663,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:36:44.359Z</v>
+        <v>2026-04-10T21:36:48.263Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data — 2026-04-10T21:36:51.303Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,28 +434,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>mp9laie6</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Launch email campaign</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>CMO</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>gtvjoxp5</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>medium</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>pending</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>Draft campaign brief</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -634,7 +634,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:36:48.263Z</v>
+        <v>2026-04-10T21:36:51.297Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KneuraCOMMS commit — 2026-04-10T21:37:52.689Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,36 +434,123 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>wsn8gzqg</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Finalize product roadmap</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>6r4bt6ge</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>high</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>in-progress</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-04-11</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>Write Q4 objectives section</v>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>0eyyjaon</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Review Q3 expense report</v>
+      </c>
+      <c r="C3" t="str">
+        <v>CFO</v>
+      </c>
+      <c r="D3" t="str">
+        <v>myftnpa4</v>
+      </c>
+      <c r="E3" t="str">
+        <v>high</v>
+      </c>
+      <c r="F3" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-04-09</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Pull receipts from Notion</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>e2w12prf</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Set up analytics dashboard</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CIO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>6r4bt6ge</v>
+      </c>
+      <c r="E4" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F4" t="str">
+        <v>blocked</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Unblock API access from vendor</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Waiting on vendor</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>bar5izig</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Launch email campaign</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CMO</v>
+      </c>
+      <c r="D5" t="str">
+        <v>6r4bt6ge</v>
+      </c>
+      <c r="E5" t="str">
+        <v>medium</v>
+      </c>
+      <c r="F5" t="str">
+        <v>pending</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Draft campaign brief</v>
+      </c>
+      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -488,7 +575,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>gtvjoxp5</v>
+        <v>6r4bt6ge</v>
       </c>
       <c r="B2" t="str">
         <v>Product Launch</v>
@@ -502,7 +589,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>fqfexnca</v>
+        <v>myftnpa4</v>
       </c>
       <c r="B3" t="str">
         <v>Q3 Financials</v>
@@ -634,7 +721,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:37:20.394Z</v>
+        <v>2026-04-10T21:37:51.987Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KneuraCOMMS commit — 2026-04-10T21:40:25.031Z
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -434,7 +434,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>wsn8gzqg</v>
+        <v>ldcr30yw</v>
       </c>
       <c r="B2" t="str">
         <v>Finalize product roadmap</v>
@@ -443,7 +443,7 @@
         <v>CEO</v>
       </c>
       <c r="D2" t="str">
-        <v>6r4bt6ge</v>
+        <v>j480qo8s</v>
       </c>
       <c r="E2" t="str">
         <v>high</v>
@@ -463,7 +463,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>0eyyjaon</v>
+        <v>sm8o6d0p</v>
       </c>
       <c r="B3" t="str">
         <v>Review Q3 expense report</v>
@@ -472,7 +472,7 @@
         <v>CFO</v>
       </c>
       <c r="D3" t="str">
-        <v>myftnpa4</v>
+        <v>ij99nlp9</v>
       </c>
       <c r="E3" t="str">
         <v>high</v>
@@ -492,7 +492,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>e2w12prf</v>
+        <v>e0tns10y</v>
       </c>
       <c r="B4" t="str">
         <v>Set up analytics dashboard</v>
@@ -501,7 +501,7 @@
         <v>CIO</v>
       </c>
       <c r="D4" t="str">
-        <v>6r4bt6ge</v>
+        <v>j480qo8s</v>
       </c>
       <c r="E4" t="str">
         <v>medium</v>
@@ -521,7 +521,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>bar5izig</v>
+        <v>u7bh46me</v>
       </c>
       <c r="B5" t="str">
         <v>Launch email campaign</v>
@@ -530,7 +530,7 @@
         <v>CMO</v>
       </c>
       <c r="D5" t="str">
-        <v>6r4bt6ge</v>
+        <v>j480qo8s</v>
       </c>
       <c r="E5" t="str">
         <v>medium</v>
@@ -575,7 +575,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>6r4bt6ge</v>
+        <v>j480qo8s</v>
       </c>
       <c r="B2" t="str">
         <v>Product Launch</v>
@@ -589,7 +589,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>myftnpa4</v>
+        <v>ij99nlp9</v>
       </c>
       <c r="B3" t="str">
         <v>Q3 Financials</v>
@@ -721,7 +721,7 @@
         <v>[]</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-10T21:37:51.987Z</v>
+        <v>2026-04-10T21:40:24.353Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data from KneuraCOMM
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -3,11 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Tasks" sheetId="1" r:id="rId1"/>
-    <sheet name="Projects" sheetId="2" r:id="rId2"/>
-    <sheet name="Payments" sheetId="3" r:id="rId3"/>
-    <sheet name="Decisions" sheetId="4" r:id="rId4"/>
-    <sheet name="Meta" sheetId="5" r:id="rId5"/>
+    <sheet name="Data" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -401,332 +397,155 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>title</v>
-      </c>
-      <c r="C1" t="str">
-        <v>role</v>
-      </c>
-      <c r="D1" t="str">
-        <v>project</v>
-      </c>
-      <c r="E1" t="str">
-        <v>priority</v>
-      </c>
-      <c r="F1" t="str">
-        <v>status</v>
-      </c>
-      <c r="G1" t="str">
-        <v>due</v>
-      </c>
-      <c r="H1" t="str">
-        <v>nextAction</v>
-      </c>
-      <c r="I1" t="str">
-        <v>notes</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ldcr30yw</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Finalize product roadmap</v>
-      </c>
-      <c r="C2" t="str">
-        <v>CEO</v>
-      </c>
-      <c r="D2" t="str">
-        <v>j480qo8s</v>
-      </c>
-      <c r="E2" t="str">
-        <v>high</v>
-      </c>
-      <c r="F2" t="str">
-        <v>in-progress</v>
-      </c>
-      <c r="G2" t="str">
-        <v>2026-04-11</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Write Q4 objectives section</v>
-      </c>
-      <c r="I2" t="str">
-        <v/>
+        <v>KneuraCOMM Data Export</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>sm8o6d0p</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Review Q3 expense report</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CFO</v>
-      </c>
-      <c r="D3" t="str">
-        <v>ij99nlp9</v>
-      </c>
-      <c r="E3" t="str">
-        <v>high</v>
-      </c>
-      <c r="F3" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G3" t="str">
-        <v>2026-04-09</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Pull receipts from Notion</v>
-      </c>
-      <c r="I3" t="str">
-        <v/>
+        <v>TASKS</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>e0tns10y</v>
+        <v>ID</v>
       </c>
       <c r="B4" t="str">
-        <v>Set up analytics dashboard</v>
+        <v>Title</v>
       </c>
       <c r="C4" t="str">
-        <v>CIO</v>
+        <v>Role</v>
       </c>
       <c r="D4" t="str">
-        <v>j480qo8s</v>
+        <v>Project</v>
       </c>
       <c r="E4" t="str">
-        <v>medium</v>
+        <v>Priority</v>
       </c>
       <c r="F4" t="str">
-        <v>blocked</v>
+        <v>Status</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-04-11</v>
+        <v>Due</v>
       </c>
       <c r="H4" t="str">
-        <v>Unblock API access from vendor</v>
+        <v>Next Action</v>
       </c>
       <c r="I4" t="str">
-        <v>Waiting on vendor</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>u7bh46me</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Launch email campaign</v>
-      </c>
-      <c r="C5" t="str">
-        <v>CMO</v>
-      </c>
-      <c r="D5" t="str">
-        <v>j480qo8s</v>
-      </c>
-      <c r="E5" t="str">
-        <v>medium</v>
-      </c>
-      <c r="F5" t="str">
-        <v>pending</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v>Draft campaign brief</v>
-      </c>
-      <c r="I5" t="str">
-        <v/>
+        <v>Estimate</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Created</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>PROJECTS</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Name</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Role</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Archived</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ixbnfoge</v>
+      </c>
+      <c r="B8" t="str">
+        <v>TerrainIntel360</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CEO</v>
+      </c>
+      <c r="D8" t="str">
+        <v>false</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PAYMENTS</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Client</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Amount</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Due</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>DECISIONS</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Timestamp</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Note</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>METADATA</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Revenue</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Revenue Auto</v>
+      </c>
+      <c r="B18" t="str">
+        <v>false</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Roles</v>
+      </c>
+      <c r="B19" t="str">
+        <v>["CEO","COO","CFO","CMO","CIO"]</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Role Colors</v>
+      </c>
+      <c r="B20" t="str">
+        <v>{}</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>role</v>
-      </c>
-      <c r="D1" t="str">
-        <v>desc</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>j480qo8s</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Product Launch</v>
-      </c>
-      <c r="C2" t="str">
-        <v>CEO</v>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>ij99nlp9</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Q3 Financials</v>
-      </c>
-      <c r="C3" t="str">
-        <v>CFO</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>client</v>
-      </c>
-      <c r="C1" t="str">
-        <v>amount</v>
-      </c>
-      <c r="D1" t="str">
-        <v>due</v>
-      </c>
-      <c r="E1" t="str">
-        <v>status</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ts</v>
-      </c>
-      <c r="B1" t="str">
-        <v>note</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>revenue</v>
-      </c>
-      <c r="B1" t="str">
-        <v>revenueAuto</v>
-      </c>
-      <c r="C1" t="str">
-        <v>roles</v>
-      </c>
-      <c r="D1" t="str">
-        <v>roleColors</v>
-      </c>
-      <c r="E1" t="str">
-        <v>archivedProjects</v>
-      </c>
-      <c r="F1" t="str">
-        <v>savedAt</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" t="str">
-        <v>false</v>
-      </c>
-      <c r="C2" t="str">
-        <v>CEO,COO,CFO,CMO,CIO</v>
-      </c>
-      <c r="D2" t="str">
-        <v>{}</v>
-      </c>
-      <c r="E2" t="str">
-        <v>[]</v>
-      </c>
-      <c r="F2" t="str">
-        <v>2026-04-10T21:40:54.133Z</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>